<commit_message>
fix: remove Kagoshima bank from list
</commit_message>
<xml_diff>
--- a/Newslist.xlsx
+++ b/Newslist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hatabe ryutarou\Desktop\Python\toybox\Toybox_for_work\ForGit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C78FA10-5C34-447D-B9D5-A5C9CC045B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{367C4486-272B-4DA3-8C8D-675FAB4B2F19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="8170" xr2:uid="{396FD7CC-7344-4B54-AEF3-0188E6E906BB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{396FD7CC-7344-4B54-AEF3-0188E6E906BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="46">
   <si>
     <t>京都銀行</t>
   </si>
@@ -98,9 +98,6 @@
     <t>清水銀行</t>
   </si>
   <si>
-    <t>鹿児島銀行</t>
-  </si>
-  <si>
     <t>https://www.kyotobank.co.jp</t>
   </si>
   <si>
@@ -146,9 +143,6 @@
     <t>https://www.nagasakibank.co.jp</t>
   </si>
   <si>
-    <t>https://www.howabank.co.jp</t>
-  </si>
-  <si>
     <t>https://www.kyogin.co.jp</t>
   </si>
   <si>
@@ -159,9 +153,6 @@
   </si>
   <si>
     <t>https://www.shimizubank.co.jp</t>
-  </si>
-  <si>
-    <t>https://www.kagin.co.jp</t>
   </si>
   <si>
     <t>name</t>
@@ -190,6 +181,10 @@
     <rPh sb="2" eb="4">
       <t>ギンコウ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.howabank.co.jp</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -653,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC7D260-B731-43BF-BB53-F2EC2CA9F031}">
-  <dimension ref="A1:D1001"/>
+  <dimension ref="A1:D1000"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="29.58203125" customWidth="1"/>
@@ -664,16 +659,16 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18.5" thickBot="1">
       <c r="A1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>45</v>
-      </c>
       <c r="D1" s="5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="18.5" thickBot="1">
@@ -681,16 +676,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C2" s="6"/>
     </row>
     <row r="3" spans="1:4" ht="18.5" thickBot="1">
       <c r="A3" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C3" s="6"/>
     </row>
@@ -699,7 +694,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" s="6"/>
     </row>
@@ -708,7 +703,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="6"/>
     </row>
@@ -717,7 +712,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" s="6"/>
     </row>
@@ -726,7 +721,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" s="6"/>
     </row>
@@ -735,7 +730,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" s="6"/>
     </row>
@@ -744,7 +739,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C9" s="6"/>
     </row>
@@ -753,7 +748,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C10" s="6"/>
     </row>
@@ -762,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" s="6"/>
     </row>
@@ -771,7 +766,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" s="6"/>
     </row>
@@ -780,7 +775,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C13" s="6"/>
     </row>
@@ -789,7 +784,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C14" s="6"/>
     </row>
@@ -798,7 +793,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C15" s="6"/>
     </row>
@@ -807,7 +802,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C16" s="6"/>
     </row>
@@ -816,7 +811,7 @@
         <v>13</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C17" s="6"/>
     </row>
@@ -825,7 +820,7 @@
         <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C18" s="6"/>
     </row>
@@ -834,7 +829,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C19" s="6"/>
     </row>
@@ -843,7 +838,7 @@
         <v>16</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C20" s="6"/>
     </row>
@@ -852,7 +847,7 @@
         <v>17</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C21" s="6"/>
     </row>
@@ -861,7 +856,7 @@
         <v>18</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C22" s="6"/>
     </row>
@@ -870,20 +865,16 @@
         <v>19</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C23" s="6"/>
     </row>
-    <row r="24" spans="1:3" ht="18.5" thickBot="1">
-      <c r="A24" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="6"/>
-    </row>
-    <row r="31" spans="1:3" ht="18.5" thickBot="1"/>
+    <row r="30" spans="1:3" ht="18.5" thickBot="1"/>
+    <row r="31" spans="1:3" ht="18.5" thickBot="1">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="7"/>
+    </row>
     <row r="32" spans="1:3" ht="18.5" thickBot="1">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
@@ -5728,11 +5719,6 @@
       <c r="A1000" s="3"/>
       <c r="B1000" s="3"/>
       <c r="C1000" s="7"/>
-    </row>
-    <row r="1001" spans="1:3" ht="18.5" thickBot="1">
-      <c r="A1001" s="3"/>
-      <c r="B1001" s="3"/>
-      <c r="C1001" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -5753,14 +5739,13 @@
     <hyperlink ref="B16" r:id="rId14" display="https://www.aichibank.co.jp/" xr:uid="{B4DC13B6-AEEE-43BA-8F39-D2F921D2916D}"/>
     <hyperlink ref="B17" r:id="rId15" display="https://www.meigin.com/" xr:uid="{E58052E9-3468-4243-949E-11E72D468457}"/>
     <hyperlink ref="B18" r:id="rId16" display="https://www.nagasakibank.co.jp/" xr:uid="{448F85E7-6A31-4A1A-A4C6-C9171417EB76}"/>
-    <hyperlink ref="B19" r:id="rId17" display="https://www.howabank.co.jp/" xr:uid="{9DF06EB9-F746-4652-8D13-1FADCFBCF985}"/>
+    <hyperlink ref="B19" r:id="rId17" xr:uid="{9DF06EB9-F746-4652-8D13-1FADCFBCF985}"/>
     <hyperlink ref="B20" r:id="rId18" display="https://www.kyogin.co.jp/" xr:uid="{67439C04-003D-4225-8224-54ACAB243B32}"/>
     <hyperlink ref="B21" r:id="rId19" display="https://www.kaiho-bank.co.jp/" xr:uid="{C7C98DDB-2268-4E6F-8705-AE9577CD183C}"/>
     <hyperlink ref="B22" r:id="rId20" display="https://www.yamanashibank.co.jp/" xr:uid="{7D2DDC68-001C-4BF8-A748-75222C3E00C4}"/>
     <hyperlink ref="B23" r:id="rId21" display="https://www.shimizubank.co.jp/" xr:uid="{A575FCA1-275C-49AE-A0FA-AACA27C0552D}"/>
-    <hyperlink ref="B24" r:id="rId22" display="https://www.kagin.co.jp/" xr:uid="{89C7EE82-A6E2-4946-BE09-0083ECAB187D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId23"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId22"/>
 </worksheet>
 </file>
</xml_diff>